<commit_message>
April 11 Current Affairs
</commit_message>
<xml_diff>
--- a/policy.xlsx
+++ b/policy.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maadh\OneDrive\Desktop\serveup\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6b78a08741e6628e/Desktop/serveup/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A0D4CDF-248A-4B1D-8615-EB7C106E6E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{4A0D4CDF-248A-4B1D-8615-EB7C106E6E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37FAAF30-D6A2-4E0D-B1B5-07478EF7BC09}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="January 2022" sheetId="3" r:id="rId1"/>
@@ -18,7 +18,8 @@
     <sheet name="April 2023" sheetId="1" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'March 2023'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'April 2023'!$A$1:$I$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'March 2023'!$A$1:$I$1</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1803" uniqueCount="1224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1875" uniqueCount="1300">
   <si>
     <t>Date</t>
   </si>
@@ -3710,6 +3711,234 @@
   </si>
   <si>
     <t>Green hydrogen holds great promise for India</t>
+  </si>
+  <si>
+    <t>Education in retreat</t>
+  </si>
+  <si>
+    <t>From 'Finlandisation' to 'Natoisation'</t>
+  </si>
+  <si>
+    <t>The institutional crisis that Pakistan faces</t>
+  </si>
+  <si>
+    <t>Varying shades of 'green'</t>
+  </si>
+  <si>
+    <t>Hydro policy in a flux</t>
+  </si>
+  <si>
+    <t>E-pharmacy regulation needs nuanced policies</t>
+  </si>
+  <si>
+    <t>An improper forum</t>
+  </si>
+  <si>
+    <t>Ministry of Truth</t>
+  </si>
+  <si>
+    <t>A broken house</t>
+  </si>
+  <si>
+    <t>Why Sri Lanka's proposed anti-terror law faces widespread criticism</t>
+  </si>
+  <si>
+    <t>The long road to women empowerment</t>
+  </si>
+  <si>
+    <t>The digital space gives wings to women entrepreneurs</t>
+  </si>
+  <si>
+    <t>Inflation versus growth: RBI's dilemma</t>
+  </si>
+  <si>
+    <t>What they don't tell you about India's poverty numbers</t>
+  </si>
+  <si>
+    <t>Cash combustion rates could separate startups</t>
+  </si>
+  <si>
+    <t>How private capital can be made to work for global public goods</t>
+  </si>
+  <si>
+    <t>MSMEs selling online need simpler GST rules</t>
+  </si>
+  <si>
+    <t>The knotty business of running cooperatives</t>
+  </si>
+  <si>
+    <t>Lessons for India from US bank debacle</t>
+  </si>
+  <si>
+    <t>Bias in higher education</t>
+  </si>
+  <si>
+    <t>ChatGPT, a double-edged weapon</t>
+  </si>
+  <si>
+    <t>Reducing inflation without raising interest rates</t>
+  </si>
+  <si>
+    <t>A potent channel</t>
+  </si>
+  <si>
+    <t>Academic freedom and the crisis in higher education</t>
+  </si>
+  <si>
+    <t>An enforced silence cannot solve India's problems</t>
+  </si>
+  <si>
+    <t>Finland's journey, from neutral to NATO</t>
+  </si>
+  <si>
+    <t>Do the wealthy influence policy-making more across all forms of democracy?</t>
+  </si>
+  <si>
+    <t>Free speech: Not Supreme Court, but the people</t>
+  </si>
+  <si>
+    <t>Too Yuan to Rock'n'Roll</t>
+  </si>
+  <si>
+    <t>Milk will spill:  Amul vs. Nandini in Namma Bengaluru</t>
+  </si>
+  <si>
+    <t>Learn from traditional farming</t>
+  </si>
+  <si>
+    <t>Setting the G20 agenda</t>
+  </si>
+  <si>
+    <t>Why we learn wrong lessons from China</t>
+  </si>
+  <si>
+    <t>The Populist Raj</t>
+  </si>
+  <si>
+    <t>Don't bet with ChatGPT</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>title</t>
+  </si>
+  <si>
+    <t>link</t>
+  </si>
+  <si>
+    <t>policy</t>
+  </si>
+  <si>
+    <t>author</t>
+  </si>
+  <si>
+    <t>brief</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1iFkMbMj1YPsBsb6afqShDORkKH9thkKW/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1rW1n1xQ2FtF4x6YzT07PN1RE2fbBZev3/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1uxTwBOe1jcI_HOUWzZhc62uMDmD5asDR/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1VbWu8whAi1zZoxEBehm-j6M0G3cbVabz/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1JMHdU3xgRiZH7xyI_ov6wbII53EXkFWD/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1v2vBDQZu-_idW29de-I0KWbPNXqoPrhr/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1fZz0CgqGbPown9PFpvJm3uwoq313w5Xx/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1W1Yg_mnIN3O3KiEo66N2PusgbJ8D0UNa/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1JLP-8pTyRcJijxsfjgX8lte0fmgQSS8q/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1ruM4yDai77pVnDXU8cyFzhOBsvbiGT8l/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/115VEO4JzZLzmGNo4NOO_H-bDq73eBCBh/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1rh62icFC2bMIS5EOiKZmRFvPRuilItDJ/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1H5YP8X96S-m3Nk17PH13pLyO79AGLfJ-/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1MDDM8vtefoT3EeFo0zdbdgzlYvhy9ZfN/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1uNpM9ubuCnwdp3d8mRdYw7jg7rK2xlSm/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1kX4b8IWdBAmLnyDVjPD5iKKYKavouDmp/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1FLcq_1rLunA52nxcuzalX4TOjF6eozqk/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1QORlQuCDtauCcP5lXdeZZ7QtgX91QS9b/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/12P737JhmqaZU9c5c0cqOIk378ZrROVDR/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1F0ETgHbuWoAnI0BdwSh9BduzFZ53vcut/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1jjy_90lFdYJE9Ct5Nc_UA61vrXCRYdRh/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/19ZAQCn_wdy3GXOR65uLlSJpumWjYYR6B/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1nAJDuYLaVmZBpL0_m38wEc4krPBH2o5P/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1rTYvody8v_SiIDjUxWrEn7PkYYVaLpAo/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1rfRCmK7xD4jcVV8CcfpAP8DIstrFE0AT/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1KwlNd576bwjhhi97fgmcT8rObnOWUeEs/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1Aw8mvPeGlL4ckk65SXM-lzMqvcTSybER/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/12WDuNzNiFqb13jvneWvMDawuVBmO9Rku/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1olyRnRyuLHbtJ93_9R9Kc4NPl7FmBFGF/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1A59YWF7Cd_OX-p2VtKjosdkXWYMJ3uPa/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1LMkKei06k9_pjGzLE1y6_hNdK-i_Ig6t/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1DOICv7GEFSoo27ET2TJQPKDNURFmY8xJ/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1vrUlgqs1bh4ndVUUHB8-PmTKiGA2-ofJ/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1DkcVjE3SXqLuCvIb7TCaJgY-0LWUKIzS/view?usp=share_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1jfvBEUckIceGdXETKIc-W8G-xMQxyWjt/view?usp=share_link</t>
   </si>
 </sst>
 </file>
@@ -3806,6 +4035,10 @@
 </file>
 
 <file path=xl/persons/person1.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
+<file path=xl/persons/person2.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
@@ -8844,7 +9077,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2031D3F6-D661-4A89-A608-6121CB87C06C}">
-  <dimension ref="A1:F329"/>
+  <dimension ref="A1:G329"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.44140625" customWidth="1"/>
@@ -8854,25 +9087,28 @@
     <col min="5" max="5" width="10.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>0</v>
+        <v>1259</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="4" t="s">
-        <v>1</v>
+        <v>1260</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>2</v>
+        <v>1264</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>5</v>
+        <v>1262</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+        <v>1263</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>1261</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>44995</v>
       </c>
@@ -8883,7 +9119,7 @@
         <v>1054</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>44995</v>
       </c>
@@ -8894,7 +9130,7 @@
         <v>1055</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>44995</v>
       </c>
@@ -8905,7 +9141,7 @@
         <v>1056</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>44995</v>
       </c>
@@ -8916,7 +9152,7 @@
         <v>1057</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>44995</v>
       </c>
@@ -8927,7 +9163,7 @@
         <v>1058</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>44995</v>
       </c>
@@ -8938,7 +9174,7 @@
         <v>1059</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>44995</v>
       </c>
@@ -8949,7 +9185,7 @@
         <v>1060</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>44995</v>
       </c>
@@ -8960,7 +9196,7 @@
         <v>1061</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>44995</v>
       </c>
@@ -8971,7 +9207,7 @@
         <v>1062</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>44995</v>
       </c>
@@ -8982,7 +9218,7 @@
         <v>1063</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>44995</v>
       </c>
@@ -8993,7 +9229,7 @@
         <v>1064</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>44995</v>
       </c>
@@ -9004,7 +9240,7 @@
         <v>1065</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>44995</v>
       </c>
@@ -9015,7 +9251,7 @@
         <v>1066</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>44995</v>
       </c>
@@ -9026,7 +9262,7 @@
         <v>1067</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>44995</v>
       </c>
@@ -12481,46 +12717,46 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1" xr:uid="{2031D3F6-D661-4A89-A608-6121CB87C06C}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F220">
-      <sortCondition ref="A1"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="A1:I1" xr:uid="{2031D3F6-D661-4A89-A608-6121CB87C06C}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F282"/>
+  <dimension ref="A1:G317"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.44140625" customWidth="1"/>
     <col min="2" max="2" width="3.33203125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="53.109375" customWidth="1"/>
-    <col min="4" max="4" width="61.21875" customWidth="1"/>
+    <col min="3" max="4" width="53.109375" customWidth="1"/>
     <col min="5" max="5" width="10.88671875" customWidth="1"/>
+    <col min="6" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="61.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>0</v>
+        <v>1259</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="4" t="s">
-        <v>1</v>
+        <v>1260</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>2</v>
+        <v>1264</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>5</v>
+        <v>1262</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+        <v>1263</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>1261</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>45017</v>
       </c>
@@ -12531,7 +12767,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>45017</v>
       </c>
@@ -12542,7 +12778,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>45017</v>
       </c>
@@ -12553,7 +12789,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>45017</v>
       </c>
@@ -12564,7 +12800,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>45017</v>
       </c>
@@ -12575,7 +12811,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>45017</v>
       </c>
@@ -12586,7 +12822,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>45017</v>
       </c>
@@ -12597,7 +12833,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>45017</v>
       </c>
@@ -12608,7 +12844,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>45017</v>
       </c>
@@ -12619,7 +12855,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>45017</v>
       </c>
@@ -12630,7 +12866,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>45017</v>
       </c>
@@ -12641,7 +12877,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>45017</v>
       </c>
@@ -12652,7 +12888,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>45017</v>
       </c>
@@ -12663,7 +12899,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>45017</v>
       </c>
@@ -12674,7 +12910,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>45017</v>
       </c>
@@ -12688,7 +12924,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>45017</v>
       </c>
@@ -12699,7 +12935,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>45017</v>
       </c>
@@ -12710,7 +12946,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>45017</v>
       </c>
@@ -12721,7 +12957,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>45017</v>
       </c>
@@ -12732,7 +12968,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>45017</v>
       </c>
@@ -12743,7 +12979,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>45017</v>
       </c>
@@ -12754,7 +12990,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>45017</v>
       </c>
@@ -12765,7 +13001,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>45017</v>
       </c>
@@ -12776,7 +13012,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>45017</v>
       </c>
@@ -12786,8 +13022,9 @@
       <c r="C25" s="3" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D25" s="3"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>45017</v>
       </c>
@@ -12798,7 +13035,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>45017</v>
       </c>
@@ -12809,7 +13046,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>45017</v>
       </c>
@@ -12820,7 +13057,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>45017</v>
       </c>
@@ -12830,8 +13067,9 @@
       <c r="C29" s="3" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D29" s="3"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>45018</v>
       </c>
@@ -12842,7 +13080,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>45018</v>
       </c>
@@ -12853,7 +13091,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>45018</v>
       </c>
@@ -15504,7 +15742,7 @@
         <v>885</v>
       </c>
     </row>
-    <row r="273" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A273" s="1">
         <v>45025</v>
       </c>
@@ -15515,7 +15753,7 @@
         <v>886</v>
       </c>
     </row>
-    <row r="274" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A274" s="1">
         <v>45025</v>
       </c>
@@ -15526,7 +15764,7 @@
         <v>887</v>
       </c>
     </row>
-    <row r="275" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A275" s="1">
         <v>45025</v>
       </c>
@@ -15537,7 +15775,7 @@
         <v>888</v>
       </c>
     </row>
-    <row r="276" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A276" s="1">
         <v>45025</v>
       </c>
@@ -15548,7 +15786,7 @@
         <v>889</v>
       </c>
     </row>
-    <row r="277" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A277" s="1">
         <v>45025</v>
       </c>
@@ -15559,7 +15797,7 @@
         <v>890</v>
       </c>
     </row>
-    <row r="278" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A278" s="1">
         <v>45025</v>
       </c>
@@ -15570,7 +15808,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="279" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A279" s="1">
         <v>45025</v>
       </c>
@@ -15581,7 +15819,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="280" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A280" s="1">
         <v>45025</v>
       </c>
@@ -15592,7 +15830,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="281" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A281" s="1">
         <v>45025</v>
       </c>
@@ -15603,7 +15841,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="282" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A282" s="1">
         <v>45025</v>
       </c>
@@ -15614,7 +15852,498 @@
         <v>895</v>
       </c>
     </row>
+    <row r="283" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A283" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B283" s="2">
+        <v>1</v>
+      </c>
+      <c r="C283" t="s">
+        <v>1224</v>
+      </c>
+      <c r="G283" t="s">
+        <v>1299</v>
+      </c>
+    </row>
+    <row r="284" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A284" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B284" s="2">
+        <v>2</v>
+      </c>
+      <c r="C284" t="s">
+        <v>1225</v>
+      </c>
+      <c r="G284" t="s">
+        <v>1298</v>
+      </c>
+    </row>
+    <row r="285" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A285" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B285" s="2">
+        <v>3</v>
+      </c>
+      <c r="C285" t="s">
+        <v>1226</v>
+      </c>
+      <c r="G285" t="s">
+        <v>1297</v>
+      </c>
+    </row>
+    <row r="286" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A286" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B286" s="2">
+        <v>4</v>
+      </c>
+      <c r="C286" t="s">
+        <v>1227</v>
+      </c>
+      <c r="G286" t="s">
+        <v>1296</v>
+      </c>
+    </row>
+    <row r="287" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A287" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B287" s="2">
+        <v>5</v>
+      </c>
+      <c r="C287" t="s">
+        <v>1228</v>
+      </c>
+      <c r="G287" t="s">
+        <v>1295</v>
+      </c>
+    </row>
+    <row r="288" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A288" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B288" s="2">
+        <v>6</v>
+      </c>
+      <c r="C288" t="s">
+        <v>1229</v>
+      </c>
+      <c r="G288" t="s">
+        <v>1294</v>
+      </c>
+    </row>
+    <row r="289" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A289" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B289" s="2">
+        <v>7</v>
+      </c>
+      <c r="C289" t="s">
+        <v>1230</v>
+      </c>
+      <c r="G289" t="s">
+        <v>1293</v>
+      </c>
+    </row>
+    <row r="290" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A290" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B290" s="2">
+        <v>8</v>
+      </c>
+      <c r="C290" t="s">
+        <v>1231</v>
+      </c>
+      <c r="G290" t="s">
+        <v>1292</v>
+      </c>
+    </row>
+    <row r="291" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A291" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B291" s="2">
+        <v>9</v>
+      </c>
+      <c r="C291" t="s">
+        <v>1232</v>
+      </c>
+      <c r="G291" t="s">
+        <v>1291</v>
+      </c>
+    </row>
+    <row r="292" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A292" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B292" s="2">
+        <v>10</v>
+      </c>
+      <c r="C292" t="s">
+        <v>1233</v>
+      </c>
+      <c r="G292" t="s">
+        <v>1290</v>
+      </c>
+    </row>
+    <row r="293" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A293" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B293" s="2">
+        <v>11</v>
+      </c>
+      <c r="C293" t="s">
+        <v>1234</v>
+      </c>
+      <c r="G293" t="s">
+        <v>1289</v>
+      </c>
+    </row>
+    <row r="294" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A294" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B294" s="2">
+        <v>12</v>
+      </c>
+      <c r="C294" t="s">
+        <v>1235</v>
+      </c>
+      <c r="G294" t="s">
+        <v>1288</v>
+      </c>
+    </row>
+    <row r="295" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A295" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B295" s="2">
+        <v>13</v>
+      </c>
+      <c r="C295" t="s">
+        <v>1236</v>
+      </c>
+      <c r="G295" t="s">
+        <v>1287</v>
+      </c>
+    </row>
+    <row r="296" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A296" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B296" s="2">
+        <v>14</v>
+      </c>
+      <c r="C296" t="s">
+        <v>1237</v>
+      </c>
+      <c r="G296" t="s">
+        <v>1286</v>
+      </c>
+    </row>
+    <row r="297" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A297" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B297" s="2">
+        <v>15</v>
+      </c>
+      <c r="C297" t="s">
+        <v>1238</v>
+      </c>
+      <c r="G297" t="s">
+        <v>1285</v>
+      </c>
+    </row>
+    <row r="298" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A298" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B298" s="2">
+        <v>16</v>
+      </c>
+      <c r="C298" t="s">
+        <v>1239</v>
+      </c>
+      <c r="G298" t="s">
+        <v>1284</v>
+      </c>
+    </row>
+    <row r="299" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A299" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B299" s="2">
+        <v>17</v>
+      </c>
+      <c r="C299" t="s">
+        <v>1240</v>
+      </c>
+      <c r="G299" t="s">
+        <v>1283</v>
+      </c>
+    </row>
+    <row r="300" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A300" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B300" s="2">
+        <v>18</v>
+      </c>
+      <c r="C300" t="s">
+        <v>1241</v>
+      </c>
+      <c r="G300" t="s">
+        <v>1282</v>
+      </c>
+    </row>
+    <row r="301" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A301" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B301" s="2">
+        <v>19</v>
+      </c>
+      <c r="C301" t="s">
+        <v>1242</v>
+      </c>
+      <c r="G301" t="s">
+        <v>1281</v>
+      </c>
+    </row>
+    <row r="302" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A302" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B302" s="2">
+        <v>20</v>
+      </c>
+      <c r="C302" t="s">
+        <v>1243</v>
+      </c>
+      <c r="G302" t="s">
+        <v>1280</v>
+      </c>
+    </row>
+    <row r="303" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A303" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B303" s="2">
+        <v>21</v>
+      </c>
+      <c r="C303" t="s">
+        <v>1244</v>
+      </c>
+      <c r="G303" t="s">
+        <v>1279</v>
+      </c>
+    </row>
+    <row r="304" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A304" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B304" s="2">
+        <v>22</v>
+      </c>
+      <c r="C304" t="s">
+        <v>1245</v>
+      </c>
+      <c r="G304" t="s">
+        <v>1278</v>
+      </c>
+    </row>
+    <row r="305" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A305" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B305" s="2">
+        <v>23</v>
+      </c>
+      <c r="C305" t="s">
+        <v>1246</v>
+      </c>
+      <c r="G305" t="s">
+        <v>1277</v>
+      </c>
+    </row>
+    <row r="306" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A306" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B306" s="2">
+        <v>24</v>
+      </c>
+      <c r="C306" t="s">
+        <v>1247</v>
+      </c>
+      <c r="G306" t="s">
+        <v>1276</v>
+      </c>
+    </row>
+    <row r="307" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A307" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B307" s="2">
+        <v>25</v>
+      </c>
+      <c r="C307" t="s">
+        <v>1248</v>
+      </c>
+      <c r="G307" t="s">
+        <v>1275</v>
+      </c>
+    </row>
+    <row r="308" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A308" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B308" s="2">
+        <v>26</v>
+      </c>
+      <c r="C308" t="s">
+        <v>1249</v>
+      </c>
+      <c r="G308" t="s">
+        <v>1274</v>
+      </c>
+    </row>
+    <row r="309" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A309" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B309" s="2">
+        <v>27</v>
+      </c>
+      <c r="C309" t="s">
+        <v>1250</v>
+      </c>
+      <c r="G309" t="s">
+        <v>1273</v>
+      </c>
+    </row>
+    <row r="310" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A310" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B310" s="2">
+        <v>28</v>
+      </c>
+      <c r="C310" t="s">
+        <v>1251</v>
+      </c>
+      <c r="G310" t="s">
+        <v>1272</v>
+      </c>
+    </row>
+    <row r="311" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A311" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B311" s="2">
+        <v>29</v>
+      </c>
+      <c r="C311" t="s">
+        <v>1252</v>
+      </c>
+      <c r="G311" t="s">
+        <v>1271</v>
+      </c>
+    </row>
+    <row r="312" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A312" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B312" s="2">
+        <v>30</v>
+      </c>
+      <c r="C312" t="s">
+        <v>1253</v>
+      </c>
+      <c r="G312" t="s">
+        <v>1270</v>
+      </c>
+    </row>
+    <row r="313" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A313" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B313" s="2">
+        <v>31</v>
+      </c>
+      <c r="C313" t="s">
+        <v>1254</v>
+      </c>
+      <c r="G313" t="s">
+        <v>1269</v>
+      </c>
+    </row>
+    <row r="314" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A314" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B314" s="2">
+        <v>32</v>
+      </c>
+      <c r="C314" t="s">
+        <v>1255</v>
+      </c>
+      <c r="G314" t="s">
+        <v>1268</v>
+      </c>
+    </row>
+    <row r="315" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A315" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B315" s="2">
+        <v>33</v>
+      </c>
+      <c r="C315" t="s">
+        <v>1256</v>
+      </c>
+      <c r="G315" t="s">
+        <v>1267</v>
+      </c>
+    </row>
+    <row r="316" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A316" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B316" s="2">
+        <v>34</v>
+      </c>
+      <c r="C316" t="s">
+        <v>1257</v>
+      </c>
+      <c r="G316" t="s">
+        <v>1266</v>
+      </c>
+    </row>
+    <row r="317" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A317" s="1">
+        <v>45027</v>
+      </c>
+      <c r="B317" s="2">
+        <v>35</v>
+      </c>
+      <c r="C317" t="s">
+        <v>1258</v>
+      </c>
+      <c r="G317" t="s">
+        <v>1265</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:I1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>